<commit_message>
testing K and H experiment
</commit_message>
<xml_diff>
--- a/Figures/Pricing/vol_comparison/example_comparison.xlsx
+++ b/Figures/Pricing/vol_comparison/example_comparison.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -442,14 +442,19 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="29" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,25 +525,50 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>std_swap_rate_at_expiry_bp</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>q05_swap_rate_at_expiry_pct</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>q50_swap_rate_at_expiry_pct</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>q95_swap_rate_at_expiry_pct</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>mean_annuity_at_expiry</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>std_annuity_at_expiry</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>actual_expiry</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>model_vol_bp</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>market_vol_bp</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>vol_error_bp</t>
         </is>
@@ -566,40 +596,55 @@
         <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>1.402754361145849</v>
+        <v>1.339043460347459</v>
       </c>
       <c r="H2" t="n">
-        <v>4.729220544687504</v>
+        <v>4.740746164559687</v>
       </c>
       <c r="I2" t="n">
-        <v>1.402754361145849</v>
+        <v>1.339043460347459</v>
       </c>
       <c r="J2" t="n">
-        <v>0.00727977496907247</v>
+        <v>0.007331708578453063</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0003503824144107792</v>
+        <v>0.000351528240578653</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>1.387492150393446</v>
+        <v>1.326722913794277</v>
       </c>
       <c r="N2" t="n">
-        <v>4.799646805852148</v>
+        <v>40.82527892558611</v>
       </c>
       <c r="O2" t="n">
+        <v>0.7128013851122026</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1.318587109953979</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2.015724277161518</v>
+      </c>
+      <c r="R2" t="n">
+        <v>4.808201047008723</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.05739551710086124</v>
+      </c>
+      <c r="T2" t="n">
         <v>1</v>
       </c>
-      <c r="P2" t="n">
-        <v>38.58498371560685</v>
-      </c>
-      <c r="Q2" t="n">
+      <c r="U2" t="n">
+        <v>38.76577101193945</v>
+      </c>
+      <c r="V2" t="n">
         <v>54.9</v>
       </c>
-      <c r="R2" t="n">
-        <v>-16.31501628439315</v>
+      <c r="W2" t="n">
+        <v>-16.13422898806055</v>
       </c>
     </row>
     <row r="3">
@@ -624,40 +669,55 @@
         <v>10</v>
       </c>
       <c r="G3" t="n">
-        <v>1.360130191240512</v>
+        <v>1.290907877790287</v>
       </c>
       <c r="H3" t="n">
-        <v>9.151234741152447</v>
+        <v>9.189135113578976</v>
       </c>
       <c r="I3" t="n">
-        <v>1.360130191240512</v>
+        <v>1.290907877790287</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01496042038065284</v>
+        <v>0.01551186529741654</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0007079710047883414</v>
+        <v>0.0007391775975867305</v>
       </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>1.370095692584202</v>
+        <v>1.310412711908555</v>
       </c>
       <c r="N3" t="n">
-        <v>9.28532795289623</v>
+        <v>41.42589245963701</v>
       </c>
       <c r="O3" t="n">
+        <v>0.6934736206195342</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1.284759100557043</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>2.031961582308978</v>
+      </c>
+      <c r="R3" t="n">
+        <v>9.315149920038749</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.1989214401645041</v>
+      </c>
+      <c r="T3" t="n">
         <v>1</v>
       </c>
-      <c r="P3" t="n">
-        <v>40.97830925249302</v>
-      </c>
-      <c r="Q3" t="n">
+      <c r="U3" t="n">
+        <v>42.31353622095975</v>
+      </c>
+      <c r="V3" t="n">
         <v>91.2</v>
       </c>
-      <c r="R3" t="n">
-        <v>-50.22169074750698</v>
+      <c r="W3" t="n">
+        <v>-48.88646377904024</v>
       </c>
     </row>
     <row r="4">
@@ -682,40 +742,55 @@
         <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>1.328791946627663</v>
+        <v>1.255059313850905</v>
       </c>
       <c r="H4" t="n">
-        <v>4.480143555611839</v>
+        <v>4.503531566613063</v>
       </c>
       <c r="I4" t="n">
-        <v>1.328791946627663</v>
+        <v>1.255059313850905</v>
       </c>
       <c r="J4" t="n">
-        <v>0.01575979306699407</v>
+        <v>0.01622842003584233</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0007180513456226681</v>
+        <v>0.0007370528652717753</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>1.353248472252962</v>
+        <v>1.29798693815905</v>
       </c>
       <c r="N4" t="n">
-        <v>4.807557030361687</v>
+        <v>91.06630530118771</v>
       </c>
       <c r="O4" t="n">
+        <v>-0.1485676586824738</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1.295092022296132</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>2.780200235411884</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.815708323664625</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.1263193030717505</v>
+      </c>
+      <c r="T4" t="n">
         <v>5</v>
       </c>
-      <c r="P4" t="n">
-        <v>39.43333539038228</v>
-      </c>
-      <c r="Q4" t="n">
+      <c r="U4" t="n">
+        <v>40.39503239246534</v>
+      </c>
+      <c r="V4" t="n">
         <v>47.99999999999999</v>
       </c>
-      <c r="R4" t="n">
-        <v>-8.566664609617721</v>
+      <c r="W4" t="n">
+        <v>-7.604967607534657</v>
       </c>
     </row>
     <row r="5">
@@ -740,40 +815,55 @@
         <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>1.320285182822001</v>
+        <v>1.248264396608786</v>
       </c>
       <c r="H5" t="n">
-        <v>8.678122935536109</v>
+        <v>8.73865385752207</v>
       </c>
       <c r="I5" t="n">
-        <v>1.320285182822001</v>
+        <v>1.248264396608786</v>
       </c>
       <c r="J5" t="n">
-        <v>0.03091246377369531</v>
+        <v>0.03233957004395811</v>
       </c>
       <c r="K5" t="n">
-        <v>0.001389329419649388</v>
+        <v>0.001459596455101639</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>1.362297950432544</v>
+        <v>1.314094133372017</v>
       </c>
       <c r="N5" t="n">
-        <v>9.309433819383131</v>
+        <v>93.65763856957182</v>
       </c>
       <c r="O5" t="n">
+        <v>-0.1525470362799135</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1.299246351143673</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2.855718395768919</v>
+      </c>
+      <c r="R5" t="n">
+        <v>9.335611398426735</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.4519245339807972</v>
+      </c>
+      <c r="T5" t="n">
         <v>5</v>
       </c>
-      <c r="P5" t="n">
-        <v>39.93123610159542</v>
-      </c>
-      <c r="Q5" t="n">
+      <c r="U5" t="n">
+        <v>41.48533835848022</v>
+      </c>
+      <c r="V5" t="n">
         <v>73.40000000000001</v>
       </c>
-      <c r="R5" t="n">
-        <v>-33.46876389840458</v>
+      <c r="W5" t="n">
+        <v>-31.91466164151978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>